<commit_message>
Corrected minor typos in analysis and REAMD files
</commit_message>
<xml_diff>
--- a/manu_sourcedata/extended_data_fig5.xlsx
+++ b/manu_sourcedata/extended_data_fig5.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manu_sourcedata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAD2D14-43CC-2F43-93A4-C7E0A8BED60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB1CA8F-F4B7-CF40-B491-B3B2C3571C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2660" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{44F82391-E562-874A-B68C-03288CBFA0D0}"/>
+    <workbookView xWindow="1400" yWindow="2340" windowWidth="27640" windowHeight="16940" activeTab="4" xr2:uid="{44F82391-E562-874A-B68C-03288CBFA0D0}"/>
   </bookViews>
   <sheets>
     <sheet name="5a" sheetId="1" r:id="rId1"/>
-    <sheet name="5b,c,d,e" sheetId="2" r:id="rId2"/>
+    <sheet name="5b" sheetId="2" r:id="rId2"/>
+    <sheet name="5c" sheetId="3" r:id="rId3"/>
+    <sheet name="5d" sheetId="4" r:id="rId4"/>
+    <sheet name="5e" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="86">
   <si>
     <t>LR</t>
   </si>
@@ -262,6 +265,39 @@
   </si>
   <si>
     <t>VEGFA_NRP1</t>
+  </si>
+  <si>
+    <t>DX_all</t>
+  </si>
+  <si>
+    <t>DX_hot</t>
+  </si>
+  <si>
+    <t>PT_all</t>
+  </si>
+  <si>
+    <t>PT_hot</t>
+  </si>
+  <si>
+    <t>Endothelial</t>
+  </si>
+  <si>
+    <t>Fibroblast</t>
+  </si>
+  <si>
+    <t>Schwann</t>
+  </si>
+  <si>
+    <t>Neuroblast</t>
+  </si>
+  <si>
+    <t>Macrophage</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>T</t>
   </si>
 </sst>
 </file>
@@ -6186,9 +6222,572 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE21088-9109-E44D-B3D1-1754FD51C79D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2">
+        <v>7.4560170190036801E-2</v>
+      </c>
+      <c r="C2">
+        <v>6.8554329361660504E-2</v>
+      </c>
+      <c r="D2">
+        <v>9.2011053363875106E-2</v>
+      </c>
+      <c r="E2">
+        <v>0.10130072826738</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3">
+        <v>0.12396856190160301</v>
+      </c>
+      <c r="C3">
+        <v>6.8810750157886694E-2</v>
+      </c>
+      <c r="D3">
+        <v>0.137090765845676</v>
+      </c>
+      <c r="E3">
+        <v>0.153594556709891</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4">
+        <v>2.3141411287096899E-2</v>
+      </c>
+      <c r="C4">
+        <v>2.1403472522398999E-2</v>
+      </c>
+      <c r="D4">
+        <v>6.8573436963366E-2</v>
+      </c>
+      <c r="E4">
+        <v>6.4694932376553493E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5">
+        <v>0.51716060987187595</v>
+      </c>
+      <c r="C5">
+        <v>0.334888440405674</v>
+      </c>
+      <c r="D5">
+        <v>0.43650765432535799</v>
+      </c>
+      <c r="E5">
+        <v>0.27791553215472697</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6">
+        <v>0.120002643925313</v>
+      </c>
+      <c r="C6">
+        <v>0.168620164267129</v>
+      </c>
+      <c r="D6">
+        <v>0.195707267968011</v>
+      </c>
+      <c r="E6">
+        <v>0.28315931200800398</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7">
+        <v>4.2030172643793703E-2</v>
+      </c>
+      <c r="C7">
+        <v>8.5188035117570601E-2</v>
+      </c>
+      <c r="D7">
+        <v>1.51163474815091E-2</v>
+      </c>
+      <c r="E7">
+        <v>1.9495973208230901E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8">
+        <v>9.9136430180279303E-2</v>
+      </c>
+      <c r="C8">
+        <v>0.25253480816767898</v>
+      </c>
+      <c r="D8">
+        <v>5.4993474052202798E-2</v>
+      </c>
+      <c r="E8">
+        <v>9.9838965275211494E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3DE9E6-6090-2E44-8317-B43457D85101}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2">
+        <v>7.4560170190036801E-2</v>
+      </c>
+      <c r="C2">
+        <v>7.5246894736910097E-2</v>
+      </c>
+      <c r="D2">
+        <v>9.2011053363875106E-2</v>
+      </c>
+      <c r="E2">
+        <v>9.0824104191554303E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3">
+        <v>0.12396856190160301</v>
+      </c>
+      <c r="C3">
+        <v>9.7122701459348301E-2</v>
+      </c>
+      <c r="D3">
+        <v>0.137090765845676</v>
+      </c>
+      <c r="E3">
+        <v>0.15706776538874201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4">
+        <v>2.3141411287096899E-2</v>
+      </c>
+      <c r="C4">
+        <v>2.6289573298789601E-2</v>
+      </c>
+      <c r="D4">
+        <v>6.8573436963366E-2</v>
+      </c>
+      <c r="E4">
+        <v>7.0302124756432993E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5">
+        <v>0.51716060987187595</v>
+      </c>
+      <c r="C5">
+        <v>0.27790551975385303</v>
+      </c>
+      <c r="D5">
+        <v>0.43650765432535799</v>
+      </c>
+      <c r="E5">
+        <v>0.178884472263101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6">
+        <v>0.120002643925313</v>
+      </c>
+      <c r="C6">
+        <v>0.19506830537476699</v>
+      </c>
+      <c r="D6">
+        <v>0.195707267968011</v>
+      </c>
+      <c r="E6">
+        <v>0.34119426712193002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7">
+        <v>4.2030172643793703E-2</v>
+      </c>
+      <c r="C7">
+        <v>8.3811879964446195E-2</v>
+      </c>
+      <c r="D7">
+        <v>1.51163474815091E-2</v>
+      </c>
+      <c r="E7">
+        <v>2.8092202092913701E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8">
+        <v>9.9136430180279303E-2</v>
+      </c>
+      <c r="C8">
+        <v>0.24455512541188501</v>
+      </c>
+      <c r="D8">
+        <v>5.4993474052202798E-2</v>
+      </c>
+      <c r="E8">
+        <v>0.133635064185324</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF491F44-23BD-EE4A-931C-425D99BA47B2}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2">
+        <v>7.4560170190036801E-2</v>
+      </c>
+      <c r="C2">
+        <v>7.8448106742018006E-2</v>
+      </c>
+      <c r="D2">
+        <v>9.2011053363875106E-2</v>
+      </c>
+      <c r="E2">
+        <v>9.6171149803407602E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3">
+        <v>0.12396856190160301</v>
+      </c>
+      <c r="C3">
+        <v>0.130811722927624</v>
+      </c>
+      <c r="D3">
+        <v>0.137090765845676</v>
+      </c>
+      <c r="E3">
+        <v>0.13582418152642201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4">
+        <v>2.3141411287096899E-2</v>
+      </c>
+      <c r="C4">
+        <v>2.6119567803173298E-2</v>
+      </c>
+      <c r="D4">
+        <v>6.8573436963366E-2</v>
+      </c>
+      <c r="E4">
+        <v>6.14662437446419E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5">
+        <v>0.51716060987187595</v>
+      </c>
+      <c r="C5">
+        <v>0.31743279995624901</v>
+      </c>
+      <c r="D5">
+        <v>0.43650765432535799</v>
+      </c>
+      <c r="E5">
+        <v>0.28196187128032502</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6">
+        <v>0.120002643925313</v>
+      </c>
+      <c r="C6">
+        <v>0.167792188279312</v>
+      </c>
+      <c r="D6">
+        <v>0.195707267968011</v>
+      </c>
+      <c r="E6">
+        <v>0.29647655977953802</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7">
+        <v>4.2030172643793703E-2</v>
+      </c>
+      <c r="C7">
+        <v>7.0343352730861397E-2</v>
+      </c>
+      <c r="D7">
+        <v>1.51163474815091E-2</v>
+      </c>
+      <c r="E7">
+        <v>2.0624460658083099E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8">
+        <v>9.9136430180279303E-2</v>
+      </c>
+      <c r="C8">
+        <v>0.20905226156076001</v>
+      </c>
+      <c r="D8">
+        <v>5.4993474052202798E-2</v>
+      </c>
+      <c r="E8">
+        <v>0.10747553320758001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C8ECDE-AC94-5046-905E-E635F9E7A97F}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2">
+        <v>7.4560170190036801E-2</v>
+      </c>
+      <c r="C2">
+        <v>7.7683849885258602E-2</v>
+      </c>
+      <c r="D2">
+        <v>9.2011053363875106E-2</v>
+      </c>
+      <c r="E2">
+        <v>9.3143599983043196E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3">
+        <v>0.12396856190160301</v>
+      </c>
+      <c r="C3">
+        <v>0.103928474592383</v>
+      </c>
+      <c r="D3">
+        <v>0.137090765845676</v>
+      </c>
+      <c r="E3">
+        <v>0.15729874411711101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4">
+        <v>2.3141411287096899E-2</v>
+      </c>
+      <c r="C4">
+        <v>2.6325205325012101E-2</v>
+      </c>
+      <c r="D4">
+        <v>6.8573436963366E-2</v>
+      </c>
+      <c r="E4">
+        <v>6.8198205055471806E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5">
+        <v>0.51716060987187595</v>
+      </c>
+      <c r="C5">
+        <v>0.27427086715555499</v>
+      </c>
+      <c r="D5">
+        <v>0.43650765432535799</v>
+      </c>
+      <c r="E5">
+        <v>0.198583076014928</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6">
+        <v>0.120002643925313</v>
+      </c>
+      <c r="C6">
+        <v>0.18914535093298701</v>
+      </c>
+      <c r="D6">
+        <v>0.195707267968011</v>
+      </c>
+      <c r="E6">
+        <v>0.32174111214169399</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7">
+        <v>4.2030172643793703E-2</v>
+      </c>
+      <c r="C7">
+        <v>8.2027464670057504E-2</v>
+      </c>
+      <c r="D7">
+        <v>1.51163474815091E-2</v>
+      </c>
+      <c r="E7">
+        <v>2.4322441507338501E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8">
+        <v>9.9136430180279303E-2</v>
+      </c>
+      <c r="C8">
+        <v>0.24661878743874499</v>
+      </c>
+      <c r="D8">
+        <v>5.4993474052202798E-2</v>
+      </c>
+      <c r="E8">
+        <v>0.136712821180411</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>